<commit_message>
fix(stability): reconnect frontend routing and regression gates
Make API/document ownership explicit, restore scoped waiver history, and exercise real query failure/refetch behavior in the complete CI suite. Start a verified UI server before browser checks and retain honest outcomes.

Refs #531, #532, #533, #534, #535, #536

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/uat/uat_master.xlsx
+++ b/docs/uat/uat_master.xlsx
@@ -3515,9 +3515,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:P190"/>
-  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="1" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns5="http://schemas.microsoft.com/office/excel/2006/main" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:P197"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="1" ns3:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="52" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
@@ -3537,7 +3537,7 @@
     <col min="16" max="16" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" ns3:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -3551,7 +3551,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" ns3:dyDescent="0.35">
       <c r="A3" s="7" t="s">
         <v>4</v>
       </c>
@@ -3601,7 +3601,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:16" ht="19" customHeight="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="A4" s="19" t="s">
         <v>20</v>
       </c>
@@ -3618,7 +3618,7 @@
       <c r="N4" s="14"/>
       <c r="O4" s="14"/>
     </row>
-    <row r="5" spans="1:16" ht="28.5" customHeight="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:16" ht="28.5" customHeight="1" outlineLevel="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="B5" s="9" t="s">
         <v>21</v>
       </c>
@@ -3654,7 +3654,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="28.5" customHeight="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:16" ht="28.5" customHeight="1" outlineLevel="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="B6" s="9" t="s">
         <v>30</v>
       </c>
@@ -3690,7 +3690,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="28.5" customHeight="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:16" ht="28.5" customHeight="1" outlineLevel="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="B7" s="9" t="s">
         <v>34</v>
       </c>
@@ -3726,7 +3726,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="28.5" customHeight="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:16" ht="28.5" customHeight="1" outlineLevel="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="B8" s="9" t="s">
         <v>38</v>
       </c>
@@ -3762,7 +3762,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="28.5" customHeight="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:16" ht="28.5" customHeight="1" outlineLevel="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="B9" s="9" t="s">
         <v>42</v>
       </c>
@@ -3798,7 +3798,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="42.5" customHeight="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:16" ht="42.5" customHeight="1" outlineLevel="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="B10" s="9" t="s">
         <v>46</v>
       </c>
@@ -3834,7 +3834,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="42.5" customHeight="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:16" ht="42.5" customHeight="1" outlineLevel="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="B11" s="9" t="s">
         <v>51</v>
       </c>
@@ -3870,7 +3870,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="42.5" customHeight="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:16" ht="42.5" customHeight="1" outlineLevel="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="B12" s="9" t="s">
         <v>55</v>
       </c>
@@ -3906,7 +3906,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:16" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" outlineLevel="1" ns3:dyDescent="0.35">
       <c r="E13" s="14"/>
       <c r="F13" s="14"/>
       <c r="H13" s="14"/>
@@ -3914,7 +3914,7 @@
       <c r="N13" s="14"/>
       <c r="O13" s="14"/>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" ns3:dyDescent="0.35">
       <c r="E14" s="14"/>
       <c r="F14" s="14"/>
       <c r="H14" s="14"/>
@@ -3922,7 +3922,7 @@
       <c r="N14" s="14"/>
       <c r="O14" s="14"/>
     </row>
-    <row r="15" spans="1:16" ht="18.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:16" ht="18.5" customHeight="1" ns3:dyDescent="0.45">
       <c r="A15" s="19" t="s">
         <v>60</v>
       </c>
@@ -3939,7 +3939,7 @@
       <c r="N15" s="14"/>
       <c r="O15" s="14"/>
     </row>
-    <row r="16" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" ht="29" ns3:dyDescent="0.35">
       <c r="B16" s="10" t="s">
         <v>61</v>
       </c>
@@ -3975,7 +3975,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="17" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:16" ht="29" ns3:dyDescent="0.35">
       <c r="B17" s="10" t="s">
         <v>67</v>
       </c>
@@ -4011,7 +4011,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="18" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:16" ht="29" ns3:dyDescent="0.35">
       <c r="B18" s="10" t="s">
         <v>71</v>
       </c>
@@ -4047,7 +4047,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="19" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:16" ht="29" ns3:dyDescent="0.35">
       <c r="B19" s="10" t="s">
         <v>76</v>
       </c>
@@ -4083,7 +4083,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="20" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:16" ht="29" ns3:dyDescent="0.35">
       <c r="B20" s="10" t="s">
         <v>80</v>
       </c>
@@ -4119,7 +4119,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="21" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:16" ht="29" ns3:dyDescent="0.35">
       <c r="B21" s="10" t="s">
         <v>85</v>
       </c>
@@ -4155,7 +4155,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="22" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:16" ht="29" ns3:dyDescent="0.35">
       <c r="B22" s="10" t="s">
         <v>89</v>
       </c>
@@ -4191,7 +4191,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="23" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:16" ht="29" ns3:dyDescent="0.35">
       <c r="B23" s="10" t="s">
         <v>93</v>
       </c>
@@ -4227,7 +4227,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:16" ht="29" ns3:dyDescent="0.35">
       <c r="B24" s="10" t="s">
         <v>97</v>
       </c>
@@ -4263,7 +4263,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="25" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:16" ht="29" ns3:dyDescent="0.35">
       <c r="B25" s="10" t="s">
         <v>101</v>
       </c>
@@ -4299,7 +4299,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="26" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:16" ht="29" ns3:dyDescent="0.35">
       <c r="B26" s="10" t="s">
         <v>106</v>
       </c>
@@ -4335,7 +4335,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="27" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:16" ht="29" ns3:dyDescent="0.35">
       <c r="B27" s="10" t="s">
         <v>111</v>
       </c>
@@ -4371,7 +4371,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:16" ht="29" ns3:dyDescent="0.35">
       <c r="B28" s="10" t="s">
         <v>115</v>
       </c>
@@ -4407,7 +4407,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="29" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:16" ht="29" ns3:dyDescent="0.35">
       <c r="B29" s="10" t="s">
         <v>119</v>
       </c>
@@ -4443,7 +4443,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="30" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:16" ht="29" ns3:dyDescent="0.35">
       <c r="B30" s="10" t="s">
         <v>123</v>
       </c>
@@ -4479,7 +4479,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="31" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:16" ht="29" ns3:dyDescent="0.35">
       <c r="B31" s="10" t="s">
         <v>127</v>
       </c>
@@ -4515,7 +4515,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="32" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:16" ht="29" ns3:dyDescent="0.35">
       <c r="B32" s="10" t="s">
         <v>131</v>
       </c>
@@ -4551,7 +4551,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:16" ns3:dyDescent="0.35">
       <c r="E33" s="14"/>
       <c r="F33" s="14"/>
       <c r="H33" s="14"/>
@@ -4559,7 +4559,7 @@
       <c r="N33" s="14"/>
       <c r="O33" s="14"/>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:16" ns3:dyDescent="0.35">
       <c r="E34" s="14"/>
       <c r="F34" s="14"/>
       <c r="H34" s="14"/>
@@ -4567,7 +4567,7 @@
       <c r="N34" s="14"/>
       <c r="O34" s="14"/>
     </row>
-    <row r="35" spans="1:16" ht="18.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:16" ht="18.5" customHeight="1" ns3:dyDescent="0.45">
       <c r="A35" s="19" t="s">
         <v>135</v>
       </c>
@@ -4584,7 +4584,7 @@
       <c r="N35" s="14"/>
       <c r="O35" s="14"/>
     </row>
-    <row r="36" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:16" ht="29" ns3:dyDescent="0.35">
       <c r="B36" s="10" t="s">
         <v>136</v>
       </c>
@@ -4620,7 +4620,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="37" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:16" ht="29" ns3:dyDescent="0.35">
       <c r="B37" s="10" t="s">
         <v>141</v>
       </c>
@@ -4656,7 +4656,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="38" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:16" ht="29" ns3:dyDescent="0.35">
       <c r="B38" s="10" t="s">
         <v>145</v>
       </c>
@@ -4692,7 +4692,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="39" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:16" ht="29" ns3:dyDescent="0.35">
       <c r="B39" s="10" t="s">
         <v>150</v>
       </c>
@@ -4728,7 +4728,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="40" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:16" ht="29" ns3:dyDescent="0.35">
       <c r="B40" s="10" t="s">
         <v>154</v>
       </c>
@@ -4764,7 +4764,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="41" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:16" ht="29" ns3:dyDescent="0.35">
       <c r="B41" s="10" t="s">
         <v>159</v>
       </c>
@@ -4800,7 +4800,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="42" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:16" ht="29" ns3:dyDescent="0.35">
       <c r="B42" s="10" t="s">
         <v>163</v>
       </c>
@@ -4836,7 +4836,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="43" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:16" ht="29" ns3:dyDescent="0.35">
       <c r="B43" s="10" t="s">
         <v>167</v>
       </c>
@@ -4872,7 +4872,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:16" ns3:dyDescent="0.35">
       <c r="B44" s="10" t="s">
         <v>171</v>
       </c>
@@ -4908,7 +4908,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:16" ns3:dyDescent="0.35">
       <c r="B45" s="10" t="s">
         <v>175</v>
       </c>
@@ -4944,7 +4944,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="46" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:16" ht="29" ns3:dyDescent="0.35">
       <c r="B46" s="10" t="s">
         <v>179</v>
       </c>
@@ -4980,7 +4980,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="47" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:16" ht="29" ns3:dyDescent="0.35">
       <c r="B47" s="10" t="s">
         <v>184</v>
       </c>
@@ -5016,7 +5016,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="48" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:16" ht="29" ns3:dyDescent="0.35">
       <c r="B48" s="10" t="s">
         <v>188</v>
       </c>
@@ -5052,7 +5052,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="49" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:16" ht="29" ns3:dyDescent="0.35">
       <c r="B49" s="10" t="s">
         <v>192</v>
       </c>
@@ -5088,7 +5088,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:16" ns3:dyDescent="0.35">
       <c r="E50" s="14"/>
       <c r="F50" s="14"/>
       <c r="H50" s="14"/>
@@ -5096,7 +5096,7 @@
       <c r="N50" s="14"/>
       <c r="O50" s="14"/>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:16" ns3:dyDescent="0.35">
       <c r="E51" s="14"/>
       <c r="F51" s="14"/>
       <c r="H51" s="14"/>
@@ -5104,7 +5104,7 @@
       <c r="N51" s="14"/>
       <c r="O51" s="14"/>
     </row>
-    <row r="52" spans="1:16" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="52" spans="1:16" ht="19" customHeight="1" thickBot="1" ns3:dyDescent="0.5">
       <c r="A52" s="19" t="s">
         <v>197</v>
       </c>
@@ -5121,7 +5121,7 @@
       <c r="N52" s="14"/>
       <c r="O52" s="14"/>
     </row>
-    <row r="53" spans="1:16" ht="42.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:16" ht="42.5" customHeight="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="A53" s="1"/>
       <c r="B53" s="9" t="s">
         <v>198</v>
@@ -5158,7 +5158,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="54" spans="1:16" ht="42.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:16" ht="42.5" customHeight="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="A54" s="1"/>
       <c r="B54" s="9" t="s">
         <v>203</v>
@@ -5195,7 +5195,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="55" spans="1:16" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:16" ht="28.5" customHeight="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="A55" s="1"/>
       <c r="B55" s="9" t="s">
         <v>207</v>
@@ -5232,7 +5232,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="56" spans="1:16" ht="42.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:16" ht="42.5" customHeight="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="A56" s="1"/>
       <c r="B56" s="9" t="s">
         <v>211</v>
@@ -5269,7 +5269,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="57" spans="1:16" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:16" ht="28.5" customHeight="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="A57" s="1"/>
       <c r="B57" s="9" t="s">
         <v>215</v>
@@ -5306,7 +5306,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="58" spans="1:16" ht="42.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:16" ht="42.5" customHeight="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="A58" s="1"/>
       <c r="B58" s="9" t="s">
         <v>219</v>
@@ -5343,7 +5343,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="59" spans="1:16" ht="42.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:16" ht="42.5" customHeight="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="A59" s="1"/>
       <c r="B59" s="9" t="s">
         <v>223</v>
@@ -5380,7 +5380,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="60" spans="1:16" ht="42.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:16" ht="42.5" customHeight="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="A60" s="1"/>
       <c r="B60" s="9" t="s">
         <v>228</v>
@@ -5417,7 +5417,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="61" spans="1:16" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:16" ht="15" customHeight="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="B61" s="9" t="s">
         <v>232</v>
       </c>
@@ -5453,7 +5453,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="62" spans="1:16" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:16" ht="15" customHeight="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="B62" s="9" t="s">
         <v>236</v>
       </c>
@@ -5489,7 +5489,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="63" spans="1:16" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:16" ht="15" customHeight="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="B63" s="9" t="s">
         <v>240</v>
       </c>
@@ -5525,7 +5525,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="64" spans="1:16" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:16" ht="15" customHeight="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="B64" s="9" t="s">
         <v>244</v>
       </c>
@@ -5561,7 +5561,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="65" spans="1:16" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:16" ht="15" customHeight="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="B65" s="9" t="s">
         <v>248</v>
       </c>
@@ -5597,7 +5597,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="66" spans="1:16" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:16" ht="15" customHeight="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="B66" s="9" t="s">
         <v>253</v>
       </c>
@@ -5633,7 +5633,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="67" spans="1:16" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:16" ht="15" customHeight="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="B67" s="9" t="s">
         <v>257</v>
       </c>
@@ -5669,7 +5669,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="68" spans="1:16" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:16" ht="15" customHeight="1" thickBot="1" ns3:dyDescent="0.4">
       <c r="B68" s="9" t="s">
         <v>262</v>
       </c>
@@ -5705,7 +5705,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="69" spans="1:16" ht="32" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:16" ht="32" ns3:dyDescent="0.35">
       <c r="A69" s="19" t="s">
         <v>266</v>
       </c>
@@ -5716,7 +5716,7 @@
       <c r="N69" s="14"/>
       <c r="O69" s="14"/>
     </row>
-    <row r="70" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:16" ht="29" ns3:dyDescent="0.35">
       <c r="B70" s="10" t="s">
         <v>267</v>
       </c>
@@ -5752,7 +5752,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="71" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:16" ht="29" ns3:dyDescent="0.35">
       <c r="B71" s="10" t="s">
         <v>272</v>
       </c>
@@ -5788,7 +5788,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="72" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:16" ht="29" ns3:dyDescent="0.35">
       <c r="B72" s="10" t="s">
         <v>276</v>
       </c>
@@ -5824,7 +5824,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="73" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:16" ht="29" ns3:dyDescent="0.35">
       <c r="B73" s="10" t="s">
         <v>280</v>
       </c>
@@ -5860,7 +5860,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="74" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:16" ht="29" ns3:dyDescent="0.35">
       <c r="B74" s="10" t="s">
         <v>286</v>
       </c>
@@ -5896,7 +5896,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="75" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:16" ht="29" ns3:dyDescent="0.35">
       <c r="B75" s="10" t="s">
         <v>291</v>
       </c>
@@ -5932,7 +5932,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="76" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:16" ht="29" ns3:dyDescent="0.35">
       <c r="B76" s="10" t="s">
         <v>297</v>
       </c>
@@ -5968,7 +5968,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="77" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:16" ht="29" ns3:dyDescent="0.35">
       <c r="B77" s="10" t="s">
         <v>301</v>
       </c>
@@ -6004,7 +6004,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="78" spans="1:16" ht="32" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:16" ht="32" ns3:dyDescent="0.35">
       <c r="A78" s="19" t="s">
         <v>306</v>
       </c>
@@ -6015,7 +6015,7 @@
       <c r="N78" s="14"/>
       <c r="O78" s="14"/>
     </row>
-    <row r="79" spans="1:16" ht="58" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:16" ht="58" ns3:dyDescent="0.35">
       <c r="B79" s="10" t="s">
         <v>307</v>
       </c>
@@ -6053,7 +6053,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="80" spans="1:16" ht="58" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:16" ht="58" ns3:dyDescent="0.35">
       <c r="B80" s="10" t="s">
         <v>314</v>
       </c>
@@ -6091,7 +6091,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="81" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B81" s="10" t="s">
         <v>318</v>
       </c>
@@ -6129,7 +6129,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="82" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B82" s="10" t="s">
         <v>323</v>
       </c>
@@ -6167,7 +6167,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="83" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B83" s="10" t="s">
         <v>326</v>
       </c>
@@ -6205,7 +6205,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="84" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B84" s="10" t="s">
         <v>331</v>
       </c>
@@ -6243,7 +6243,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="85" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B85" s="10" t="s">
         <v>334</v>
       </c>
@@ -6281,7 +6281,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="86" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B86" s="10" t="s">
         <v>339</v>
       </c>
@@ -6319,7 +6319,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="87" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B87" s="10" t="s">
         <v>342</v>
       </c>
@@ -6357,7 +6357,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="88" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B88" s="10" t="s">
         <v>348</v>
       </c>
@@ -6395,7 +6395,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="89" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B89" s="10" t="s">
         <v>352</v>
       </c>
@@ -6433,7 +6433,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="90" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B90" s="10" t="s">
         <v>357</v>
       </c>
@@ -6471,7 +6471,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="91" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B91" s="10" t="s">
         <v>359</v>
       </c>
@@ -6509,7 +6509,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="92" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B92" s="10" t="s">
         <v>362</v>
       </c>
@@ -6547,7 +6547,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="93" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B93" s="10" t="s">
         <v>364</v>
       </c>
@@ -6585,7 +6585,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="94" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B94" s="10" t="s">
         <v>367</v>
       </c>
@@ -6623,7 +6623,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="95" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B95" s="10" t="s">
         <v>369</v>
       </c>
@@ -6661,7 +6661,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="96" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B96" s="10" t="s">
         <v>372</v>
       </c>
@@ -6699,7 +6699,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="97" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B97" s="10" t="s">
         <v>374</v>
       </c>
@@ -6737,7 +6737,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="98" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B98" s="10" t="s">
         <v>377</v>
       </c>
@@ -6775,7 +6775,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="99" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B99" s="10" t="s">
         <v>379</v>
       </c>
@@ -6813,7 +6813,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="100" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B100" s="10" t="s">
         <v>382</v>
       </c>
@@ -6851,7 +6851,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="101" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B101" s="10" t="s">
         <v>384</v>
       </c>
@@ -6889,7 +6889,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="102" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B102" s="10" t="s">
         <v>389</v>
       </c>
@@ -6927,7 +6927,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="103" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B103" s="10" t="s">
         <v>391</v>
       </c>
@@ -6965,7 +6965,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="104" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B104" s="10" t="s">
         <v>396</v>
       </c>
@@ -7003,7 +7003,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="105" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B105" s="10" t="s">
         <v>398</v>
       </c>
@@ -7041,7 +7041,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="106" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B106" s="10" t="s">
         <v>403</v>
       </c>
@@ -7079,7 +7079,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="107" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B107" s="10" t="s">
         <v>405</v>
       </c>
@@ -7117,7 +7117,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="108" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B108" s="10" t="s">
         <v>410</v>
       </c>
@@ -7155,7 +7155,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="109" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B109" s="10" t="s">
         <v>412</v>
       </c>
@@ -7193,7 +7193,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="110" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B110" s="10" t="s">
         <v>417</v>
       </c>
@@ -7231,7 +7231,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="111" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B111" s="10" t="s">
         <v>419</v>
       </c>
@@ -7269,7 +7269,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="112" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B112" s="10" t="s">
         <v>422</v>
       </c>
@@ -7307,7 +7307,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="113" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B113" s="10" t="s">
         <v>424</v>
       </c>
@@ -7345,7 +7345,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="114" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B114" s="10" t="s">
         <v>429</v>
       </c>
@@ -7383,7 +7383,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="115" spans="2:16" ht="58" x14ac:dyDescent="0.35">
+    <row r="115" spans="2:16" ht="58" ns3:dyDescent="0.35">
       <c r="B115" s="10" t="s">
         <v>431</v>
       </c>
@@ -7421,7 +7421,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="116" spans="2:16" ht="58" x14ac:dyDescent="0.35">
+    <row r="116" spans="2:16" ht="58" ns3:dyDescent="0.35">
       <c r="B116" s="10" t="s">
         <v>436</v>
       </c>
@@ -7459,7 +7459,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="117" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="117" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B117" s="10" t="s">
         <v>438</v>
       </c>
@@ -7497,7 +7497,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="118" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="118" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B118" s="10" t="s">
         <v>443</v>
       </c>
@@ -7535,7 +7535,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="119" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="119" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B119" s="10" t="s">
         <v>446</v>
       </c>
@@ -7573,7 +7573,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="120" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="120" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B120" s="10" t="s">
         <v>451</v>
       </c>
@@ -7611,7 +7611,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="121" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="121" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B121" s="10" t="s">
         <v>454</v>
       </c>
@@ -7649,7 +7649,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="122" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="122" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B122" s="10" t="s">
         <v>459</v>
       </c>
@@ -7687,7 +7687,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="123" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="123" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B123" s="10" t="s">
         <v>462</v>
       </c>
@@ -7725,7 +7725,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="124" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="124" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B124" s="10" t="s">
         <v>467</v>
       </c>
@@ -7763,7 +7763,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="125" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="125" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B125" s="10" t="s">
         <v>470</v>
       </c>
@@ -7801,7 +7801,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="126" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="126" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B126" s="10" t="s">
         <v>475</v>
       </c>
@@ -7839,7 +7839,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="127" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="127" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B127" s="10" t="s">
         <v>478</v>
       </c>
@@ -7877,7 +7877,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="128" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="128" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B128" s="10" t="s">
         <v>483</v>
       </c>
@@ -7915,7 +7915,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="129" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="129" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B129" s="10" t="s">
         <v>486</v>
       </c>
@@ -7953,7 +7953,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="130" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="130" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B130" s="10" t="s">
         <v>491</v>
       </c>
@@ -7991,7 +7991,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="131" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="131" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B131" s="10" t="s">
         <v>494</v>
       </c>
@@ -8029,7 +8029,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="132" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="132" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B132" s="10" t="s">
         <v>499</v>
       </c>
@@ -8067,7 +8067,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="133" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="133" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B133" s="10" t="s">
         <v>502</v>
       </c>
@@ -8105,7 +8105,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="134" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="134" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B134" s="10" t="s">
         <v>507</v>
       </c>
@@ -8143,7 +8143,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="135" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="135" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B135" s="10" t="s">
         <v>510</v>
       </c>
@@ -8181,7 +8181,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="136" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="136" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B136" s="10" t="s">
         <v>515</v>
       </c>
@@ -8219,7 +8219,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="137" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="137" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B137" s="10" t="s">
         <v>518</v>
       </c>
@@ -8257,7 +8257,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="138" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="138" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B138" s="10" t="s">
         <v>523</v>
       </c>
@@ -8295,7 +8295,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="139" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="139" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B139" s="10" t="s">
         <v>526</v>
       </c>
@@ -8333,7 +8333,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="140" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="140" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B140" s="10" t="s">
         <v>529</v>
       </c>
@@ -8371,7 +8371,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="141" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="141" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B141" s="10" t="s">
         <v>531</v>
       </c>
@@ -8409,7 +8409,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="142" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="142" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B142" s="10" t="s">
         <v>536</v>
       </c>
@@ -8447,7 +8447,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="143" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="143" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B143" s="10" t="s">
         <v>539</v>
       </c>
@@ -8485,7 +8485,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="144" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="144" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B144" s="10" t="s">
         <v>544</v>
       </c>
@@ -8523,7 +8523,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="145" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B145" s="10" t="s">
         <v>547</v>
       </c>
@@ -8561,7 +8561,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="146" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B146" s="10" t="s">
         <v>552</v>
       </c>
@@ -8599,7 +8599,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="147" spans="1:16" ht="32" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:16" ht="32" ns3:dyDescent="0.35">
       <c r="A147" s="19" t="s">
         <v>556</v>
       </c>
@@ -8610,7 +8610,7 @@
       <c r="N147" s="14"/>
       <c r="O147" s="14"/>
     </row>
-    <row r="148" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B148" s="10" t="s">
         <v>557</v>
       </c>
@@ -8648,7 +8648,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="149" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B149" s="10" t="s">
         <v>563</v>
       </c>
@@ -8686,7 +8686,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="150" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B150" s="10" t="s">
         <v>568</v>
       </c>
@@ -8724,7 +8724,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="151" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B151" s="10" t="s">
         <v>573</v>
       </c>
@@ -8762,7 +8762,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="152" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:16" ht="72.5" ns3:dyDescent="0.35">
       <c r="B152" s="10" t="s">
         <v>578</v>
       </c>
@@ -8800,7 +8800,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="153" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B153" s="10" t="s">
         <v>583</v>
       </c>
@@ -8838,7 +8838,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="154" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B154" s="10" t="s">
         <v>588</v>
       </c>
@@ -8876,7 +8876,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="155" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B155" s="10" t="s">
         <v>593</v>
       </c>
@@ -8914,7 +8914,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="156" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B156" s="10" t="s">
         <v>598</v>
       </c>
@@ -8952,7 +8952,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="157" spans="1:16" ht="58" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:16" ht="58" ns3:dyDescent="0.35">
       <c r="B157" s="10" t="s">
         <v>603</v>
       </c>
@@ -8990,7 +8990,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="158" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B158" s="10" t="s">
         <v>608</v>
       </c>
@@ -9028,7 +9028,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="159" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B159" s="10" t="s">
         <v>613</v>
       </c>
@@ -9066,7 +9066,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="160" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B160" s="10" t="s">
         <v>618</v>
       </c>
@@ -9104,7 +9104,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="161" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="161" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B161" s="10" t="s">
         <v>623</v>
       </c>
@@ -9142,7 +9142,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="162" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="162" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B162" s="10" t="s">
         <v>628</v>
       </c>
@@ -9180,7 +9180,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="163" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="163" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B163" s="10" t="s">
         <v>633</v>
       </c>
@@ -9218,7 +9218,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="164" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="164" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B164" s="10" t="s">
         <v>638</v>
       </c>
@@ -9256,7 +9256,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="165" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="165" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B165" s="10" t="s">
         <v>643</v>
       </c>
@@ -9294,7 +9294,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="166" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="166" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B166" s="10" t="s">
         <v>648</v>
       </c>
@@ -9332,7 +9332,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="167" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="167" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B167" s="10" t="s">
         <v>653</v>
       </c>
@@ -9370,7 +9370,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="168" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="168" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B168" s="10" t="s">
         <v>658</v>
       </c>
@@ -9408,7 +9408,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="169" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="169" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B169" s="10" t="s">
         <v>663</v>
       </c>
@@ -9446,7 +9446,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="170" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="170" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B170" s="10" t="s">
         <v>668</v>
       </c>
@@ -9484,7 +9484,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="171" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="171" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B171" s="10" t="s">
         <v>673</v>
       </c>
@@ -9522,7 +9522,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="172" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="172" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B172" s="10" t="s">
         <v>678</v>
       </c>
@@ -9560,7 +9560,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="173" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="173" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B173" s="10" t="s">
         <v>683</v>
       </c>
@@ -9598,7 +9598,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="174" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="174" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B174" s="10" t="s">
         <v>688</v>
       </c>
@@ -9636,7 +9636,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="175" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="175" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B175" s="10" t="s">
         <v>693</v>
       </c>
@@ -9674,7 +9674,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="176" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="176" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B176" s="10" t="s">
         <v>698</v>
       </c>
@@ -9712,7 +9712,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="177" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="177" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B177" s="10" t="s">
         <v>703</v>
       </c>
@@ -9750,7 +9750,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="178" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="178" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B178" s="10" t="s">
         <v>708</v>
       </c>
@@ -9788,7 +9788,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="179" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="179" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B179" s="10" t="s">
         <v>713</v>
       </c>
@@ -9826,7 +9826,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="180" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="180" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B180" s="10" t="s">
         <v>718</v>
       </c>
@@ -9864,7 +9864,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="181" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="181" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B181" s="10" t="s">
         <v>723</v>
       </c>
@@ -9902,7 +9902,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="182" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="182" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B182" s="10" t="s">
         <v>728</v>
       </c>
@@ -9940,7 +9940,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="183" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="183" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B183" s="10" t="s">
         <v>733</v>
       </c>
@@ -9978,7 +9978,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="184" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="184" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B184" s="10" t="s">
         <v>738</v>
       </c>
@@ -10016,7 +10016,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="185" spans="2:16" ht="58" x14ac:dyDescent="0.35">
+    <row r="185" spans="2:16" ht="58" ns3:dyDescent="0.35">
       <c r="B185" s="10" t="s">
         <v>743</v>
       </c>
@@ -10054,7 +10054,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="186" spans="2:16" ht="58" x14ac:dyDescent="0.35">
+    <row r="186" spans="2:16" ht="58" ns3:dyDescent="0.35">
       <c r="B186" s="10" t="s">
         <v>747</v>
       </c>
@@ -10092,7 +10092,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="187" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="187" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B187" s="10" t="s">
         <v>751</v>
       </c>
@@ -10130,7 +10130,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="188" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="188" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B188" s="10" t="s">
         <v>755</v>
       </c>
@@ -10168,7 +10168,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="189" spans="2:16" ht="58" x14ac:dyDescent="0.35">
+    <row r="189" spans="2:16" ht="58" ns3:dyDescent="0.35">
       <c r="B189" s="10" t="s">
         <v>759</v>
       </c>
@@ -10206,7 +10206,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="190" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="190" spans="2:16" ht="43.5" ns3:dyDescent="0.35">
       <c r="B190" s="10" t="s">
         <v>763</v>
       </c>
@@ -10242,6 +10242,460 @@
       </c>
       <c r="P190" s="29" t="s">
         <v>285</v>
+      </c>
+    </row>
+    <row r="191" spans="1:16" ns3:dyDescent="0.35">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Commissioner waiver history - stability and recovery regression</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="192" spans="2:16" ht="58" ns3:dyDescent="0.35">
+      <c r="B192" s="10" t="inlineStr">
+        <is>
+          <t>6.69</t>
+        </is>
+      </c>
+      <c r="C192" s="24" t="inlineStr">
+        <is>
+          <t>Commissioner &gt; Manage Waiver Rules</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E192" s="25" t="inlineStr">
+        <is>
+          <t>Open Commissioner &gt; Manage Waiver Rules in a league with completed claims, then refresh the page.</t>
+        </is>
+      </c>
+      <c r="F192" s="26" t="inlineStr">
+        <is>
+          <t>The claim history shows the selected league's completed claims and remains correct after refresh.</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="H192" s="14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J192" s="14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>Commissioner</t>
+        </is>
+      </c>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>TRC-STABILITY-6.69</t>
+        </is>
+      </c>
+      <c r="N192" s="14" t="inlineStr">
+        <is>
+          <t>https://github.com/NPGrant81/fantasy-football-pi/issues/534</t>
+        </is>
+      </c>
+      <c r="O192" s="14" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/commissioner/ManageWaiverRules.jsx</t>
+        </is>
+      </c>
+      <c r="P192" s="29" t="inlineStr">
+        <is>
+          <t>P0 - Critical Path</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" spans="2:16" ht="58" ns3:dyDescent="0.35">
+      <c r="B193" s="10" t="inlineStr">
+        <is>
+          <t>6.70</t>
+        </is>
+      </c>
+      <c r="C193" s="24" t="inlineStr">
+        <is>
+          <t>Commissioner &gt; Manage Waiver Rules</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E193" s="25" t="inlineStr">
+        <is>
+          <t>Open Commissioner &gt; Manage Waiver Rules in a league with no claims.</t>
+        </is>
+      </c>
+      <c r="F193" s="26" t="inlineStr">
+        <is>
+          <t>The history shows no claims, without an error or claims from another league.</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="H193" s="14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J193" s="14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>Commissioner</t>
+        </is>
+      </c>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>TRC-STABILITY-6.70</t>
+        </is>
+      </c>
+      <c r="N193" s="14" t="inlineStr">
+        <is>
+          <t>https://github.com/NPGrant81/fantasy-football-pi/issues/534</t>
+        </is>
+      </c>
+      <c r="O193" s="14" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/commissioner/ManageWaiverRules.jsx</t>
+        </is>
+      </c>
+      <c r="P193" s="29" t="inlineStr">
+        <is>
+          <t>P1 - Core Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" spans="2:16" ht="58" ns3:dyDescent="0.35">
+      <c r="B194" s="10" t="inlineStr">
+        <is>
+          <t>6.71</t>
+        </is>
+      </c>
+      <c r="C194" s="24" t="inlineStr">
+        <is>
+          <t>Commissioner &gt; Manage Waiver Rules</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E194" s="25" t="inlineStr">
+        <is>
+          <t>With QA simulating a temporary history-loading failure, open Manage Waiver Rules. Restore access and select Retry waiver history.</t>
+        </is>
+      </c>
+      <c r="F194" s="26" t="inlineStr">
+        <is>
+          <t>A clear error appears instead of empty success. Retry loads the claim history after access is restored.</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="H194" s="14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J194" s="14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>Commissioner</t>
+        </is>
+      </c>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>TRC-STABILITY-6.71</t>
+        </is>
+      </c>
+      <c r="N194" s="14" t="inlineStr">
+        <is>
+          <t>https://github.com/NPGrant81/fantasy-football-pi/issues/534</t>
+        </is>
+      </c>
+      <c r="O194" s="14" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/commissioner/ManageWaiverRules.jsx</t>
+        </is>
+      </c>
+      <c r="P194" s="29" t="inlineStr">
+        <is>
+          <t>P1 - Core Regression</t>
+        </is>
+      </c>
+    </row>
+    <row r="195" spans="2:16" ht="58" ns3:dyDescent="0.35">
+      <c r="B195" s="10" t="inlineStr">
+        <is>
+          <t>6.72</t>
+        </is>
+      </c>
+      <c r="C195" s="24" t="inlineStr">
+        <is>
+          <t>Commissioner &gt; Manage Waiver Rules</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E195" s="25" t="inlineStr">
+        <is>
+          <t>With QA restricting history access, open Manage Waiver Rules and try Retry waiver history.</t>
+        </is>
+      </c>
+      <c r="F195" s="26" t="inlineStr">
+        <is>
+          <t>A clear permission message remains visible and no restricted claims are displayed.</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="H195" s="14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J195" s="14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>Commissioner</t>
+        </is>
+      </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>TRC-STABILITY-6.72</t>
+        </is>
+      </c>
+      <c r="N195" s="14" t="inlineStr">
+        <is>
+          <t>https://github.com/NPGrant81/fantasy-football-pi/issues/534</t>
+        </is>
+      </c>
+      <c r="O195" s="14" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/commissioner/ManageWaiverRules.jsx</t>
+        </is>
+      </c>
+      <c r="P195" s="29" t="inlineStr">
+        <is>
+          <t>P0 - Critical Path</t>
+        </is>
+      </c>
+    </row>
+    <row r="196" spans="2:16" ht="58" ns3:dyDescent="0.35">
+      <c r="B196" s="10" t="inlineStr">
+        <is>
+          <t>6.73</t>
+        </is>
+      </c>
+      <c r="C196" s="24" t="inlineStr">
+        <is>
+          <t>Commissioner &gt; Manage Waiver Rules</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E196" s="25" t="inlineStr">
+        <is>
+          <t>Delay loading the first league's history with QA, switch to another league, then allow both loads to finish.</t>
+        </is>
+      </c>
+      <c r="F196" s="26" t="inlineStr">
+        <is>
+          <t>Only the newly selected league's history appears; the delayed first league does not replace it.</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="H196" s="14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J196" s="14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>Commissioner</t>
+        </is>
+      </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>TRC-STABILITY-6.73</t>
+        </is>
+      </c>
+      <c r="N196" s="14" t="inlineStr">
+        <is>
+          <t>https://github.com/NPGrant81/fantasy-football-pi/issues/534</t>
+        </is>
+      </c>
+      <c r="O196" s="14" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/commissioner/ManageWaiverRules.jsx</t>
+        </is>
+      </c>
+      <c r="P196" s="29" t="inlineStr">
+        <is>
+          <t>P0 - Critical Path</t>
+        </is>
+      </c>
+    </row>
+    <row r="197" spans="2:16" ht="58" ns3:dyDescent="0.35">
+      <c r="B197" s="10" t="inlineStr">
+        <is>
+          <t>6.74</t>
+        </is>
+      </c>
+      <c r="C197" s="24" t="inlineStr">
+        <is>
+          <t>Commissioner &gt; Manage Waiver Rules</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E197" s="25" t="inlineStr">
+        <is>
+          <t>Open Commissioner &gt; Manage Waiver Rules directly in a new tab, then refresh the page.</t>
+        </is>
+      </c>
+      <c r="F197" s="26" t="inlineStr">
+        <is>
+          <t>The app page loads normally and claim history is either shown or reports a clear, retryable error.</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>Not Tested</t>
+        </is>
+      </c>
+      <c r="H197" s="14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J197" s="14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>Commissioner</t>
+        </is>
+      </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>TRC-STABILITY-6.74</t>
+        </is>
+      </c>
+      <c r="N197" s="14" t="inlineStr">
+        <is>
+          <t>https://github.com/NPGrant81/fantasy-football-pi/issues/532</t>
+        </is>
+      </c>
+      <c r="O197" s="14" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/commissioner/ManageWaiverRules.jsx</t>
+        </is>
+      </c>
+      <c r="P197" s="29" t="inlineStr">
+        <is>
+          <t>P1 - Core Regression</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -10336,39 +10790,39 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="5">
-        <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000000000000}">
-          <x14:formula1>
-            <xm:f>Dropdown_Lists!$A$1:$A$5</xm:f>
-          </x14:formula1>
-          <xm:sqref>G5:G2000</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000001000000}">
-          <x14:formula1>
-            <xm:f>Dropdown_Lists!$B$1:$B$4</xm:f>
-          </x14:formula1>
-          <xm:sqref>I5:I2000</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
-          <x14:formula1>
-            <xm:f>Dropdown_Lists!$C$1:$C$4</xm:f>
-          </x14:formula1>
-          <xm:sqref>K5:K2000</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000003000000}">
-          <x14:formula1>
-            <xm:f>Dropdown_Lists!$D$1:$D$4</xm:f>
-          </x14:formula1>
-          <xm:sqref>L5:L2000</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0000-000004000000}">
-          <x14:formula1>
-            <xm:f>Dropdown_Lists!$G$2:$G$4</xm:f>
-          </x14:formula1>
-          <xm:sqref>P5:P2000</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
+    <ext uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <ns4:dataValidations count="5">
+        <ns4:dataValidation type="list" allowBlank="1" ns2:uid="{00000000-0002-0000-0000-000000000000}">
+          <ns4:formula1>
+            <ns5:f>Dropdown_Lists!$A$1:$A$5</ns5:f>
+          </ns4:formula1>
+          <ns5:sqref>G5:G2000</ns5:sqref>
+        </ns4:dataValidation>
+        <ns4:dataValidation type="list" allowBlank="1" ns2:uid="{00000000-0002-0000-0000-000001000000}">
+          <ns4:formula1>
+            <ns5:f>Dropdown_Lists!$B$1:$B$4</ns5:f>
+          </ns4:formula1>
+          <ns5:sqref>I5:I2000</ns5:sqref>
+        </ns4:dataValidation>
+        <ns4:dataValidation type="list" allowBlank="1" ns2:uid="{00000000-0002-0000-0000-000002000000}">
+          <ns4:formula1>
+            <ns5:f>Dropdown_Lists!$C$1:$C$4</ns5:f>
+          </ns4:formula1>
+          <ns5:sqref>K5:K2000</ns5:sqref>
+        </ns4:dataValidation>
+        <ns4:dataValidation type="list" allowBlank="1" ns2:uid="{00000000-0002-0000-0000-000003000000}">
+          <ns4:formula1>
+            <ns5:f>Dropdown_Lists!$D$1:$D$4</ns5:f>
+          </ns4:formula1>
+          <ns5:sqref>L5:L2000</ns5:sqref>
+        </ns4:dataValidation>
+        <ns4:dataValidation type="list" allowBlank="1" ns2:uid="{00000000-0002-0000-0000-000004000000}">
+          <ns4:formula1>
+            <ns5:f>Dropdown_Lists!$G$2:$G$4</ns5:f>
+          </ns4:formula1>
+          <ns5:sqref>P5:P2000</ns5:sqref>
+        </ns4:dataValidation>
+      </ns4:dataValidations>
     </ext>
   </extLst>
 </worksheet>

</xml_diff>